<commit_message>
feat(goat): add DMA breakout discovery scanner
Broad daily scan across S&P 500 + ASX 200 for names whose close just
crossed above their 150-day or 200-day MA (checked independently, no
base pattern, no rising-sector filter, slope informational only) --
distinct from Heartbeat Scan's compound entry signal and Monitor's
holdings-only downside 150DMA exit check. Ethical filter, liquidity/
market-cap floor, and fundamentals survival-context insolvency
suppression gate staging into goat_pending_candidates.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/investments/share_profit_target_calculator.xlsx
+++ b/investments/share_profit_target_calculator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\AI\Dynamous\Courses\second-brain-workshop\investments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3184FDE7-C380-439C-80BC-CBAB5D0E556A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC9B0079-0AC1-4E62-9EEB-5DC28B9A1A7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -493,7 +493,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="3">
-        <v>500</v>
+        <v>900</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -510,7 +510,7 @@
       </c>
       <c r="B12" s="7">
         <f>(B5*B6+B7+B8+B9)/B5</f>
-        <v>9.48</v>
+        <v>10.28</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -519,7 +519,7 @@
       </c>
       <c r="B13" s="4">
         <f>B12*B5</f>
-        <v>4740</v>
+        <v>5140</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -537,7 +537,7 @@
       </c>
       <c r="B15" s="4">
         <f>B13-B14-B8</f>
-        <v>500</v>
+        <v>900</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -571,7 +571,7 @@
       </c>
       <c r="B20" s="4">
         <f>B19-B9</f>
-        <v>925</v>
+        <v>525</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
feat: add Matt Damon Price/Volatility/Volume Check to my-trader; archive completed plans
Adds a new my-trader assessment check (checks/matt_damon_price_volitility_volume_check.py)
that reads price/volatility/volume rate-of-change together over short (10d) and
long (25d) windows, wired unconditionally into engine.py so it appears in both
Monitor's daily report and find --ticker. Ships as verdict="info" only -- the
alignment label is descriptive, not a validated predictive claim -- until the
companion one-off backtest script (matt_damon_price_volitility_volume_check_backtest.py,
run via the new `matt-damon-backtest` CLI subcommand) checks it against real
holdings/watchlist history.

Also archives 10 completed .agent/plans/*.md files into .agent/plans/completed/,
and picks up incidental local edits (paste-shortcuts.md, share_profit_target_calculator.xlsx).
</commit_message>
<xml_diff>
--- a/investments/share_profit_target_calculator.xlsx
+++ b/investments/share_profit_target_calculator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\AI\Dynamous\Courses\second-brain-workshop\investments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC9B0079-0AC1-4E62-9EEB-5DC28B9A1A7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DE07A50-453B-4AE3-99F2-FA2E596E5AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -461,7 +461,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2">
-        <v>500</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -469,7 +469,7 @@
         <v>18</v>
       </c>
       <c r="B6" s="3">
-        <v>8.48</v>
+        <v>5.86</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -493,7 +493,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="3">
-        <v>900</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -510,7 +510,7 @@
       </c>
       <c r="B12" s="7">
         <f>(B5*B6+B7+B8+B9)/B5</f>
-        <v>10.28</v>
+        <v>6.16</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -519,7 +519,7 @@
       </c>
       <c r="B13" s="4">
         <f>B12*B5</f>
-        <v>5140</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -528,7 +528,7 @@
       </c>
       <c r="B14" s="4">
         <f>B5*B6+B7</f>
-        <v>4240</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -537,7 +537,7 @@
       </c>
       <c r="B15" s="4">
         <f>B13-B14-B8</f>
-        <v>900</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -553,7 +553,7 @@
         <v>14</v>
       </c>
       <c r="B18" s="5">
-        <v>11.33</v>
+        <v>6.14</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -562,7 +562,7 @@
       </c>
       <c r="B19" s="4">
         <f>B18*B5-B14-B8</f>
-        <v>1425</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -571,7 +571,7 @@
       </c>
       <c r="B20" s="4">
         <f>B19-B9</f>
-        <v>525</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>